<commit_message>
edits for new input sheets
</commit_message>
<xml_diff>
--- a/STN_EMULATOR/Output/20260623/All_PTM_ECOPTM_Event_Horizon_Results.xlsx
+++ b/STN_EMULATOR/Output/20260623/All_PTM_ECOPTM_Event_Horizon_Results.xlsx
@@ -8,15 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lamanuel\Documents\github\STN_emulator_dashboard\STN_EMULATOR\Output\20260623\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B06BE39B-1FBC-42CB-9CB2-62E0C3D412D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{546F22B2-2067-4A97-AA6C-EA87B38A0285}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
-    <workbookView xWindow="6045" yWindow="3810" windowWidth="21600" windowHeight="11295" xr2:uid="{78069E8D-D483-4ECD-8D19-2B9A30F7E01D}"/>
+    <workbookView xWindow="7260" yWindow="0" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Scenario_Inputs" sheetId="1" r:id="rId1"/>
-    <sheet name="Combined_Model_Results" sheetId="2" r:id="rId2"/>
-    <sheet name="PTM_All_Scenarios" sheetId="3" r:id="rId3"/>
+    <sheet name="Combined_Results" sheetId="2" r:id="rId2"/>
+    <sheet name="PTM_Results" sheetId="3" r:id="rId3"/>
     <sheet name="ECO_PTM_Results" sheetId="4" r:id="rId4"/>
     <sheet name="Event_Horizon_Results" sheetId="5" r:id="rId5"/>
     <sheet name="Dummy_Input_Notes" sheetId="6" r:id="rId6"/>
@@ -48,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3060" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3130" uniqueCount="146">
   <si>
     <t>Scenario</t>
   </si>
@@ -470,13 +469,22 @@
     <t>Link to dl</t>
   </si>
   <si>
-    <t>Forecast_scenario</t>
+    <t>Forecast average</t>
   </si>
   <si>
-    <t>PTM_scenario</t>
+    <t>Historic 30-day average</t>
   </si>
   <si>
-    <t>baseline</t>
+    <t>Historic 7-day average</t>
+  </si>
+  <si>
+    <t>Emulator_Scenario</t>
+  </si>
+  <si>
+    <t>Historic</t>
+  </si>
+  <si>
+    <t>OMRI -3500</t>
   </si>
 </sst>
 </file>
@@ -3869,7 +3877,7 @@
   <sheetData>
     <row r="1" spans="1:21" s="1" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="18" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B1" s="19" t="s">
         <v>1</v>
@@ -3881,7 +3889,7 @@
         <v>3</v>
       </c>
       <c r="E1" s="19" t="s">
-        <v>140</v>
+        <v>0</v>
       </c>
       <c r="F1" s="19" t="s">
         <v>29</v>
@@ -3934,7 +3942,7 @@
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A2" s="15" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="B2" s="16">
         <v>46195</v>
@@ -3945,8 +3953,8 @@
       <c r="D2" s="15">
         <v>7</v>
       </c>
-      <c r="E2" s="15">
-        <v>-3500</v>
+      <c r="E2" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="F2" s="17" t="s">
         <v>37</v>
@@ -3995,7 +4003,7 @@
     </row>
     <row r="3" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="B3" s="12">
         <v>46195</v>
@@ -4006,8 +4014,8 @@
       <c r="D3" s="8">
         <v>7</v>
       </c>
-      <c r="E3" s="15">
-        <v>-3500</v>
+      <c r="E3" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="F3" s="9" t="s">
         <v>41</v>
@@ -4056,7 +4064,7 @@
     </row>
     <row r="4" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="B4" s="12">
         <v>46195</v>
@@ -4067,8 +4075,8 @@
       <c r="D4" s="8">
         <v>7</v>
       </c>
-      <c r="E4" s="15">
-        <v>-3500</v>
+      <c r="E4" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="F4" s="9" t="s">
         <v>43</v>
@@ -4119,7 +4127,7 @@
     </row>
     <row r="5" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="B5" s="12">
         <v>46195</v>
@@ -4130,8 +4138,8 @@
       <c r="D5" s="8">
         <v>7</v>
       </c>
-      <c r="E5" s="15">
-        <v>-3500</v>
+      <c r="E5" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="F5" s="9" t="s">
         <v>43</v>
@@ -4182,7 +4190,7 @@
     </row>
     <row r="6" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="B6" s="12">
         <v>46195</v>
@@ -4193,8 +4201,8 @@
       <c r="D6" s="8">
         <v>7</v>
       </c>
-      <c r="E6" s="15">
-        <v>-3500</v>
+      <c r="E6" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="F6" s="9" t="s">
         <v>43</v>
@@ -4245,7 +4253,7 @@
     </row>
     <row r="7" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="B7" s="12">
         <v>46195</v>
@@ -4256,8 +4264,8 @@
       <c r="D7" s="8">
         <v>7</v>
       </c>
-      <c r="E7" s="15">
-        <v>-3500</v>
+      <c r="E7" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="F7" s="9" t="s">
         <v>43</v>
@@ -4308,7 +4316,7 @@
     </row>
     <row r="8" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="B8" s="12">
         <v>46195</v>
@@ -4319,8 +4327,8 @@
       <c r="D8" s="8">
         <v>7</v>
       </c>
-      <c r="E8" s="15">
-        <v>-3500</v>
+      <c r="E8" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="F8" s="9" t="s">
         <v>43</v>
@@ -4371,7 +4379,7 @@
     </row>
     <row r="9" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="B9" s="12">
         <v>46195</v>
@@ -4382,8 +4390,8 @@
       <c r="D9" s="8">
         <v>7</v>
       </c>
-      <c r="E9" s="15">
-        <v>-3500</v>
+      <c r="E9" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="F9" s="9" t="s">
         <v>43</v>
@@ -4434,7 +4442,7 @@
     </row>
     <row r="10" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="B10" s="12">
         <v>46195</v>
@@ -4445,8 +4453,8 @@
       <c r="D10" s="8">
         <v>7</v>
       </c>
-      <c r="E10" s="15">
-        <v>-3500</v>
+      <c r="E10" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="F10" s="9" t="s">
         <v>43</v>
@@ -4497,7 +4505,7 @@
     </row>
     <row r="11" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="B11" s="12">
         <v>46195</v>
@@ -4508,8 +4516,8 @@
       <c r="D11" s="8">
         <v>7</v>
       </c>
-      <c r="E11" s="15">
-        <v>-3500</v>
+      <c r="E11" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="F11" s="9" t="s">
         <v>43</v>
@@ -4560,7 +4568,7 @@
     </row>
     <row r="12" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="B12" s="12">
         <v>46195</v>
@@ -4571,8 +4579,8 @@
       <c r="D12" s="8">
         <v>7</v>
       </c>
-      <c r="E12" s="15">
-        <v>-3500</v>
+      <c r="E12" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="F12" s="9" t="s">
         <v>43</v>
@@ -4623,7 +4631,7 @@
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="B13" s="12">
         <v>46195</v>
@@ -4634,8 +4642,8 @@
       <c r="D13" s="8">
         <v>7</v>
       </c>
-      <c r="E13" s="15">
-        <v>-3500</v>
+      <c r="E13" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="F13" s="9" t="s">
         <v>43</v>
@@ -4686,7 +4694,7 @@
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="B14" s="12">
         <v>46195</v>
@@ -4697,8 +4705,8 @@
       <c r="D14" s="8">
         <v>7</v>
       </c>
-      <c r="E14" s="15">
-        <v>-3500</v>
+      <c r="E14" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="F14" s="9" t="s">
         <v>43</v>
@@ -4749,7 +4757,7 @@
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="B15" s="12">
         <v>46195</v>
@@ -4760,8 +4768,8 @@
       <c r="D15" s="8">
         <v>7</v>
       </c>
-      <c r="E15" s="15">
-        <v>-3500</v>
+      <c r="E15" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="F15" s="9" t="s">
         <v>43</v>
@@ -4812,7 +4820,7 @@
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="B16" s="12">
         <v>46195</v>
@@ -4823,8 +4831,8 @@
       <c r="D16" s="8">
         <v>7</v>
       </c>
-      <c r="E16" s="15">
-        <v>-3500</v>
+      <c r="E16" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="F16" s="9" t="s">
         <v>43</v>
@@ -4875,7 +4883,7 @@
     </row>
     <row r="17" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="B17" s="12">
         <v>46195</v>
@@ -4886,8 +4894,8 @@
       <c r="D17" s="8">
         <v>7</v>
       </c>
-      <c r="E17" s="15">
-        <v>-3500</v>
+      <c r="E17" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="F17" s="9" t="s">
         <v>43</v>
@@ -4938,7 +4946,7 @@
     </row>
     <row r="18" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="B18" s="12">
         <v>46195</v>
@@ -4949,8 +4957,8 @@
       <c r="D18" s="8">
         <v>7</v>
       </c>
-      <c r="E18" s="15">
-        <v>-3500</v>
+      <c r="E18" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="F18" s="9" t="s">
         <v>47</v>
@@ -5001,7 +5009,7 @@
     </row>
     <row r="19" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="B19" s="12">
         <v>46195</v>
@@ -5012,8 +5020,8 @@
       <c r="D19" s="8">
         <v>7</v>
       </c>
-      <c r="E19" s="15">
-        <v>-3500</v>
+      <c r="E19" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="F19" s="9" t="s">
         <v>47</v>
@@ -5064,7 +5072,7 @@
     </row>
     <row r="20" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="B20" s="12">
         <v>46195</v>
@@ -5075,8 +5083,8 @@
       <c r="D20" s="8">
         <v>7</v>
       </c>
-      <c r="E20" s="15">
-        <v>-3500</v>
+      <c r="E20" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="F20" s="9" t="s">
         <v>47</v>
@@ -5127,7 +5135,7 @@
     </row>
     <row r="21" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="B21" s="12">
         <v>46195</v>
@@ -5138,8 +5146,8 @@
       <c r="D21" s="8">
         <v>7</v>
       </c>
-      <c r="E21" s="15">
-        <v>-3500</v>
+      <c r="E21" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="F21" s="9" t="s">
         <v>47</v>
@@ -5190,7 +5198,7 @@
     </row>
     <row r="22" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A22" s="8" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="B22" s="12">
         <v>46195</v>
@@ -5201,8 +5209,8 @@
       <c r="D22" s="8">
         <v>7</v>
       </c>
-      <c r="E22" s="15">
-        <v>-3500</v>
+      <c r="E22" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="F22" s="9" t="s">
         <v>47</v>
@@ -5253,7 +5261,7 @@
     </row>
     <row r="23" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A23" s="8" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="B23" s="12">
         <v>46195</v>
@@ -5264,8 +5272,8 @@
       <c r="D23" s="8">
         <v>7</v>
       </c>
-      <c r="E23" s="15">
-        <v>-3500</v>
+      <c r="E23" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="F23" s="9" t="s">
         <v>47</v>
@@ -5316,7 +5324,7 @@
     </row>
     <row r="24" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A24" s="8" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="B24" s="12">
         <v>46195</v>
@@ -5327,8 +5335,8 @@
       <c r="D24" s="8">
         <v>7</v>
       </c>
-      <c r="E24" s="15">
-        <v>-3500</v>
+      <c r="E24" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="F24" s="9" t="s">
         <v>47</v>
@@ -5379,7 +5387,7 @@
     </row>
     <row r="25" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A25" s="8" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="B25" s="12">
         <v>46195</v>
@@ -5390,8 +5398,8 @@
       <c r="D25" s="8">
         <v>7</v>
       </c>
-      <c r="E25" s="15">
-        <v>-3500</v>
+      <c r="E25" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="F25" s="9" t="s">
         <v>47</v>
@@ -5442,7 +5450,7 @@
     </row>
     <row r="26" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A26" s="8" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="B26" s="12">
         <v>46195</v>
@@ -5453,8 +5461,8 @@
       <c r="D26" s="8">
         <v>7</v>
       </c>
-      <c r="E26" s="15">
-        <v>-3500</v>
+      <c r="E26" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="F26" s="9" t="s">
         <v>47</v>
@@ -5505,7 +5513,7 @@
     </row>
     <row r="27" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A27" s="8" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="B27" s="12">
         <v>46195</v>
@@ -5516,8 +5524,8 @@
       <c r="D27" s="8">
         <v>7</v>
       </c>
-      <c r="E27" s="15">
-        <v>-3500</v>
+      <c r="E27" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="F27" s="9" t="s">
         <v>47</v>
@@ -5568,7 +5576,7 @@
     </row>
     <row r="28" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A28" s="8" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="B28" s="12">
         <v>46195</v>
@@ -5579,8 +5587,8 @@
       <c r="D28" s="8">
         <v>7</v>
       </c>
-      <c r="E28" s="15">
-        <v>-3500</v>
+      <c r="E28" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="F28" s="9" t="s">
         <v>47</v>
@@ -5631,7 +5639,7 @@
     </row>
     <row r="29" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A29" s="8" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="B29" s="12">
         <v>46195</v>
@@ -5642,8 +5650,8 @@
       <c r="D29" s="8">
         <v>7</v>
       </c>
-      <c r="E29" s="15">
-        <v>-3500</v>
+      <c r="E29" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="F29" s="9" t="s">
         <v>47</v>
@@ -5694,7 +5702,7 @@
     </row>
     <row r="30" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A30" s="8" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="B30" s="12">
         <v>46195</v>
@@ -5705,8 +5713,8 @@
       <c r="D30" s="8">
         <v>7</v>
       </c>
-      <c r="E30" s="15">
-        <v>-3500</v>
+      <c r="E30" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="F30" s="9" t="s">
         <v>47</v>
@@ -5757,7 +5765,7 @@
     </row>
     <row r="31" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A31" s="8" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="B31" s="12">
         <v>46195</v>
@@ -5768,8 +5776,8 @@
       <c r="D31" s="8">
         <v>7</v>
       </c>
-      <c r="E31" s="15">
-        <v>-3500</v>
+      <c r="E31" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="F31" s="9" t="s">
         <v>47</v>
@@ -5820,7 +5828,7 @@
     </row>
     <row r="32" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A32" s="8" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="B32" s="12">
         <v>46195</v>
@@ -5831,8 +5839,8 @@
       <c r="D32" s="8">
         <v>7</v>
       </c>
-      <c r="E32" s="15">
-        <v>-3500</v>
+      <c r="E32" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="F32" s="9" t="s">
         <v>47</v>
@@ -5883,7 +5891,7 @@
     </row>
     <row r="33" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A33" s="8" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="B33" s="12">
         <v>46195</v>
@@ -5894,8 +5902,8 @@
       <c r="D33" s="8">
         <v>7</v>
       </c>
-      <c r="E33" s="15">
-        <v>-3500</v>
+      <c r="E33" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="F33" s="9" t="s">
         <v>47</v>
@@ -5946,7 +5954,7 @@
     </row>
     <row r="34" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A34" s="8" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="B34" s="12">
         <v>46195</v>
@@ -5957,8 +5965,8 @@
       <c r="D34" s="8">
         <v>7</v>
       </c>
-      <c r="E34" s="15">
-        <v>-3500</v>
+      <c r="E34" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="F34" s="9" t="s">
         <v>47</v>
@@ -6009,7 +6017,7 @@
     </row>
     <row r="35" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A35" s="8" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="B35" s="12">
         <v>46195</v>
@@ -6020,8 +6028,8 @@
       <c r="D35" s="8">
         <v>7</v>
       </c>
-      <c r="E35" s="15">
-        <v>-3500</v>
+      <c r="E35" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="F35" s="9" t="s">
         <v>47</v>
@@ -6072,7 +6080,7 @@
     </row>
     <row r="36" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A36" s="8" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="B36" s="12">
         <v>46195</v>
@@ -6083,8 +6091,8 @@
       <c r="D36" s="8">
         <v>7</v>
       </c>
-      <c r="E36" s="15">
-        <v>-3500</v>
+      <c r="E36" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="F36" s="9" t="s">
         <v>47</v>
@@ -6135,7 +6143,7 @@
     </row>
     <row r="37" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A37" s="8" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="B37" s="12">
         <v>46195</v>
@@ -6146,8 +6154,8 @@
       <c r="D37" s="8">
         <v>7</v>
       </c>
-      <c r="E37" s="15">
-        <v>-3500</v>
+      <c r="E37" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="F37" s="9" t="s">
         <v>47</v>
@@ -6198,7 +6206,7 @@
     </row>
     <row r="38" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A38" s="8" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="B38" s="12">
         <v>46195</v>
@@ -6209,8 +6217,8 @@
       <c r="D38" s="8">
         <v>7</v>
       </c>
-      <c r="E38" s="15">
-        <v>-3500</v>
+      <c r="E38" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="F38" s="9" t="s">
         <v>47</v>
@@ -6261,7 +6269,7 @@
     </row>
     <row r="39" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A39" s="8" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="B39" s="12">
         <v>46195</v>
@@ -6272,8 +6280,8 @@
       <c r="D39" s="8">
         <v>7</v>
       </c>
-      <c r="E39" s="15">
-        <v>-3500</v>
+      <c r="E39" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="F39" s="9" t="s">
         <v>47</v>
@@ -6324,7 +6332,7 @@
     </row>
     <row r="40" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A40" s="8" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="B40" s="12">
         <v>46195</v>
@@ -6335,8 +6343,8 @@
       <c r="D40" s="8">
         <v>7</v>
       </c>
-      <c r="E40" s="15">
-        <v>-3500</v>
+      <c r="E40" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="F40" s="9" t="s">
         <v>47</v>
@@ -6387,7 +6395,7 @@
     </row>
     <row r="41" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A41" s="8" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="B41" s="12">
         <v>46195</v>
@@ -6398,8 +6406,8 @@
       <c r="D41" s="8">
         <v>7</v>
       </c>
-      <c r="E41" s="15">
-        <v>-3500</v>
+      <c r="E41" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="F41" s="9" t="s">
         <v>47</v>
@@ -6450,7 +6458,7 @@
     </row>
     <row r="42" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A42" s="8" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="B42" s="12">
         <v>46195</v>
@@ -6461,8 +6469,8 @@
       <c r="D42" s="8">
         <v>7</v>
       </c>
-      <c r="E42" s="15">
-        <v>-3500</v>
+      <c r="E42" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="F42" s="9" t="s">
         <v>47</v>
@@ -6513,7 +6521,7 @@
     </row>
     <row r="43" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A43" s="8" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="B43" s="12">
         <v>46195</v>
@@ -6524,8 +6532,8 @@
       <c r="D43" s="8">
         <v>7</v>
       </c>
-      <c r="E43" s="15">
-        <v>-3500</v>
+      <c r="E43" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="F43" s="9" t="s">
         <v>47</v>
@@ -6576,7 +6584,7 @@
     </row>
     <row r="44" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A44" s="8" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="B44" s="12">
         <v>46195</v>
@@ -6587,8 +6595,8 @@
       <c r="D44" s="8">
         <v>7</v>
       </c>
-      <c r="E44" s="15">
-        <v>-3500</v>
+      <c r="E44" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="F44" s="9" t="s">
         <v>47</v>
@@ -6639,7 +6647,7 @@
     </row>
     <row r="45" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A45" s="8" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="B45" s="12">
         <v>46195</v>
@@ -6650,8 +6658,8 @@
       <c r="D45" s="8">
         <v>7</v>
       </c>
-      <c r="E45" s="15">
-        <v>-3500</v>
+      <c r="E45" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="F45" s="9" t="s">
         <v>47</v>
@@ -6702,7 +6710,7 @@
     </row>
     <row r="46" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A46" s="8" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="B46" s="12">
         <v>46195</v>
@@ -6713,8 +6721,8 @@
       <c r="D46" s="8">
         <v>7</v>
       </c>
-      <c r="E46" s="15">
-        <v>-3500</v>
+      <c r="E46" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="F46" s="9" t="s">
         <v>47</v>
@@ -6765,7 +6773,7 @@
     </row>
     <row r="47" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A47" s="8" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="B47" s="12">
         <v>46195</v>
@@ -6776,8 +6784,8 @@
       <c r="D47" s="8">
         <v>7</v>
       </c>
-      <c r="E47" s="15">
-        <v>-3500</v>
+      <c r="E47" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="F47" s="9" t="s">
         <v>47</v>
@@ -6828,7 +6836,7 @@
     </row>
     <row r="48" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A48" s="8" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="B48" s="12">
         <v>46195</v>
@@ -6839,8 +6847,8 @@
       <c r="D48" s="8">
         <v>7</v>
       </c>
-      <c r="E48" s="15">
-        <v>-3500</v>
+      <c r="E48" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="F48" s="9" t="s">
         <v>47</v>
@@ -6891,7 +6899,7 @@
     </row>
     <row r="49" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A49" s="8" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="B49" s="12">
         <v>46195</v>
@@ -6902,8 +6910,8 @@
       <c r="D49" s="8">
         <v>7</v>
       </c>
-      <c r="E49" s="15">
-        <v>-3500</v>
+      <c r="E49" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="F49" s="9" t="s">
         <v>47</v>
@@ -6954,7 +6962,7 @@
     </row>
     <row r="50" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A50" s="8" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="B50" s="12">
         <v>46195</v>
@@ -6965,8 +6973,8 @@
       <c r="D50" s="8">
         <v>7</v>
       </c>
-      <c r="E50" s="15">
-        <v>-3500</v>
+      <c r="E50" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="F50" s="9" t="s">
         <v>47</v>
@@ -7017,7 +7025,7 @@
     </row>
     <row r="51" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A51" s="8" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="B51" s="12">
         <v>46195</v>
@@ -7028,8 +7036,8 @@
       <c r="D51" s="8">
         <v>7</v>
       </c>
-      <c r="E51" s="15">
-        <v>-3500</v>
+      <c r="E51" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="F51" s="9" t="s">
         <v>47</v>
@@ -7080,7 +7088,7 @@
     </row>
     <row r="52" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A52" s="8" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="B52" s="12">
         <v>46195</v>
@@ -7091,8 +7099,8 @@
       <c r="D52" s="8">
         <v>7</v>
       </c>
-      <c r="E52" s="15">
-        <v>-3500</v>
+      <c r="E52" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="F52" s="9" t="s">
         <v>47</v>
@@ -7143,7 +7151,7 @@
     </row>
     <row r="53" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A53" s="8" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="B53" s="12">
         <v>46195</v>
@@ -7154,8 +7162,8 @@
       <c r="D53" s="8">
         <v>7</v>
       </c>
-      <c r="E53" s="15">
-        <v>-3500</v>
+      <c r="E53" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="F53" s="9" t="s">
         <v>47</v>
@@ -7206,7 +7214,7 @@
     </row>
     <row r="54" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A54" s="8" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="B54" s="12">
         <v>46195</v>
@@ -7217,8 +7225,8 @@
       <c r="D54" s="8">
         <v>7</v>
       </c>
-      <c r="E54" s="15">
-        <v>-3500</v>
+      <c r="E54" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="F54" s="9" t="s">
         <v>47</v>
@@ -7269,7 +7277,7 @@
     </row>
     <row r="55" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A55" s="8" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="B55" s="12">
         <v>46195</v>
@@ -7280,8 +7288,8 @@
       <c r="D55" s="8">
         <v>7</v>
       </c>
-      <c r="E55" s="15">
-        <v>-3500</v>
+      <c r="E55" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="F55" s="9" t="s">
         <v>47</v>
@@ -7332,7 +7340,7 @@
     </row>
     <row r="56" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A56" s="8" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="B56" s="12">
         <v>46195</v>
@@ -7343,8 +7351,8 @@
       <c r="D56" s="8">
         <v>7</v>
       </c>
-      <c r="E56" s="15">
-        <v>-3500</v>
+      <c r="E56" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="F56" s="9" t="s">
         <v>47</v>
@@ -7395,7 +7403,7 @@
     </row>
     <row r="57" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A57" s="8" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="B57" s="12">
         <v>46195</v>
@@ -7406,8 +7414,8 @@
       <c r="D57" s="8">
         <v>7</v>
       </c>
-      <c r="E57" s="15">
-        <v>-3500</v>
+      <c r="E57" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="F57" s="9" t="s">
         <v>50</v>
@@ -7458,7 +7466,7 @@
     </row>
     <row r="58" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A58" s="8" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="B58" s="12">
         <v>46195</v>
@@ -7469,8 +7477,8 @@
       <c r="D58" s="8">
         <v>7</v>
       </c>
-      <c r="E58" s="15">
-        <v>-3500</v>
+      <c r="E58" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="F58" s="9" t="s">
         <v>50</v>
@@ -7521,7 +7529,7 @@
     </row>
     <row r="59" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A59" s="8" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="B59" s="12">
         <v>46195</v>
@@ -7532,8 +7540,8 @@
       <c r="D59" s="8">
         <v>7</v>
       </c>
-      <c r="E59" s="15">
-        <v>-3500</v>
+      <c r="E59" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="F59" s="9" t="s">
         <v>50</v>
@@ -7584,7 +7592,7 @@
     </row>
     <row r="60" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A60" s="8" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="B60" s="12">
         <v>46195</v>
@@ -7595,8 +7603,8 @@
       <c r="D60" s="8">
         <v>7</v>
       </c>
-      <c r="E60" s="15">
-        <v>-3500</v>
+      <c r="E60" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="F60" s="9" t="s">
         <v>50</v>
@@ -7647,7 +7655,7 @@
     </row>
     <row r="61" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A61" s="8" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="B61" s="12">
         <v>46195</v>
@@ -7658,8 +7666,8 @@
       <c r="D61" s="8">
         <v>7</v>
       </c>
-      <c r="E61" s="15">
-        <v>-3500</v>
+      <c r="E61" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="F61" s="9" t="s">
         <v>50</v>
@@ -7710,7 +7718,7 @@
     </row>
     <row r="62" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A62" s="8" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="B62" s="12">
         <v>46195</v>
@@ -7721,8 +7729,8 @@
       <c r="D62" s="8">
         <v>7</v>
       </c>
-      <c r="E62" s="15">
-        <v>-3500</v>
+      <c r="E62" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="F62" s="9" t="s">
         <v>50</v>
@@ -7773,7 +7781,7 @@
     </row>
     <row r="63" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A63" s="8" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="B63" s="12">
         <v>46195</v>
@@ -7784,8 +7792,8 @@
       <c r="D63" s="8">
         <v>7</v>
       </c>
-      <c r="E63" s="15">
-        <v>-3500</v>
+      <c r="E63" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="F63" s="9" t="s">
         <v>50</v>
@@ -7836,7 +7844,7 @@
     </row>
     <row r="64" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A64" s="8" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="B64" s="12">
         <v>46195</v>
@@ -7847,8 +7855,8 @@
       <c r="D64" s="8">
         <v>7</v>
       </c>
-      <c r="E64" s="15">
-        <v>-3500</v>
+      <c r="E64" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="F64" s="9" t="s">
         <v>50</v>
@@ -7899,7 +7907,7 @@
     </row>
     <row r="65" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A65" s="8" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="B65" s="12">
         <v>46195</v>
@@ -7910,8 +7918,8 @@
       <c r="D65" s="8">
         <v>7</v>
       </c>
-      <c r="E65" s="15">
-        <v>-3500</v>
+      <c r="E65" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="F65" s="9" t="s">
         <v>50</v>
@@ -7962,7 +7970,7 @@
     </row>
     <row r="66" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A66" s="8" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="B66" s="12">
         <v>46195</v>
@@ -7973,8 +7981,8 @@
       <c r="D66" s="8">
         <v>7</v>
       </c>
-      <c r="E66" s="15">
-        <v>-3500</v>
+      <c r="E66" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="F66" s="9" t="s">
         <v>50</v>
@@ -8025,7 +8033,7 @@
     </row>
     <row r="67" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A67" s="8" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="B67" s="12">
         <v>46195</v>
@@ -8036,8 +8044,8 @@
       <c r="D67" s="8">
         <v>7</v>
       </c>
-      <c r="E67" s="15">
-        <v>-3500</v>
+      <c r="E67" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="F67" s="9" t="s">
         <v>50</v>
@@ -8088,7 +8096,7 @@
     </row>
     <row r="68" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A68" s="8" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="B68" s="12">
         <v>46195</v>
@@ -8099,8 +8107,8 @@
       <c r="D68" s="8">
         <v>7</v>
       </c>
-      <c r="E68" s="15">
-        <v>-3500</v>
+      <c r="E68" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="F68" s="9" t="s">
         <v>50</v>
@@ -8151,7 +8159,7 @@
     </row>
     <row r="69" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A69" s="8" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="B69" s="12">
         <v>46195</v>
@@ -8162,8 +8170,8 @@
       <c r="D69" s="8">
         <v>7</v>
       </c>
-      <c r="E69" s="15">
-        <v>-3500</v>
+      <c r="E69" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="F69" s="9" t="s">
         <v>50</v>
@@ -8214,7 +8222,7 @@
     </row>
     <row r="70" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A70" s="8" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="B70" s="12">
         <v>46195</v>
@@ -8225,8 +8233,8 @@
       <c r="D70" s="8">
         <v>7</v>
       </c>
-      <c r="E70" s="15">
-        <v>-3500</v>
+      <c r="E70" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="F70" s="9" t="s">
         <v>50</v>
@@ -8277,7 +8285,7 @@
     </row>
     <row r="71" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A71" s="8" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="B71" s="12">
         <v>46195</v>
@@ -8288,8 +8296,8 @@
       <c r="D71" s="8">
         <v>7</v>
       </c>
-      <c r="E71" s="15">
-        <v>-3500</v>
+      <c r="E71" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="F71" s="9" t="s">
         <v>50</v>
@@ -8340,7 +8348,7 @@
     </row>
     <row r="72" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A72" s="10" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B72" s="13">
         <v>46165</v>
@@ -8352,7 +8360,7 @@
         <v>30</v>
       </c>
       <c r="E72" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F72" s="9" t="s">
         <v>37</v>
@@ -8401,7 +8409,7 @@
     </row>
     <row r="73" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A73" s="10" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B73" s="13">
         <v>46165</v>
@@ -8413,7 +8421,7 @@
         <v>30</v>
       </c>
       <c r="E73" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F73" s="9" t="s">
         <v>41</v>
@@ -8462,7 +8470,7 @@
     </row>
     <row r="74" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A74" s="10" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B74" s="13">
         <v>46165</v>
@@ -8474,7 +8482,7 @@
         <v>30</v>
       </c>
       <c r="E74" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F74" s="9" t="s">
         <v>43</v>
@@ -8525,7 +8533,7 @@
     </row>
     <row r="75" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A75" s="10" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B75" s="13">
         <v>46165</v>
@@ -8537,7 +8545,7 @@
         <v>30</v>
       </c>
       <c r="E75" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F75" s="9" t="s">
         <v>43</v>
@@ -8588,7 +8596,7 @@
     </row>
     <row r="76" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A76" s="10" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B76" s="13">
         <v>46165</v>
@@ -8600,7 +8608,7 @@
         <v>30</v>
       </c>
       <c r="E76" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F76" s="9" t="s">
         <v>43</v>
@@ -8651,7 +8659,7 @@
     </row>
     <row r="77" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A77" s="10" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B77" s="13">
         <v>46165</v>
@@ -8663,7 +8671,7 @@
         <v>30</v>
       </c>
       <c r="E77" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F77" s="9" t="s">
         <v>43</v>
@@ -8714,7 +8722,7 @@
     </row>
     <row r="78" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A78" s="10" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B78" s="13">
         <v>46165</v>
@@ -8726,7 +8734,7 @@
         <v>30</v>
       </c>
       <c r="E78" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F78" s="9" t="s">
         <v>43</v>
@@ -8777,7 +8785,7 @@
     </row>
     <row r="79" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A79" s="10" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B79" s="13">
         <v>46165</v>
@@ -8789,7 +8797,7 @@
         <v>30</v>
       </c>
       <c r="E79" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F79" s="9" t="s">
         <v>43</v>
@@ -8840,7 +8848,7 @@
     </row>
     <row r="80" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A80" s="10" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B80" s="13">
         <v>46165</v>
@@ -8852,7 +8860,7 @@
         <v>30</v>
       </c>
       <c r="E80" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F80" s="9" t="s">
         <v>43</v>
@@ -8903,7 +8911,7 @@
     </row>
     <row r="81" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A81" s="10" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B81" s="13">
         <v>46165</v>
@@ -8915,7 +8923,7 @@
         <v>30</v>
       </c>
       <c r="E81" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F81" s="9" t="s">
         <v>43</v>
@@ -8966,7 +8974,7 @@
     </row>
     <row r="82" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A82" s="10" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B82" s="13">
         <v>46165</v>
@@ -8978,7 +8986,7 @@
         <v>30</v>
       </c>
       <c r="E82" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F82" s="9" t="s">
         <v>43</v>
@@ -9029,7 +9037,7 @@
     </row>
     <row r="83" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A83" s="10" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B83" s="13">
         <v>46165</v>
@@ -9041,7 +9049,7 @@
         <v>30</v>
       </c>
       <c r="E83" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F83" s="9" t="s">
         <v>43</v>
@@ -9092,7 +9100,7 @@
     </row>
     <row r="84" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A84" s="10" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B84" s="13">
         <v>46165</v>
@@ -9104,7 +9112,7 @@
         <v>30</v>
       </c>
       <c r="E84" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F84" s="9" t="s">
         <v>43</v>
@@ -9155,7 +9163,7 @@
     </row>
     <row r="85" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A85" s="10" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B85" s="13">
         <v>46165</v>
@@ -9167,7 +9175,7 @@
         <v>30</v>
       </c>
       <c r="E85" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F85" s="9" t="s">
         <v>43</v>
@@ -9218,7 +9226,7 @@
     </row>
     <row r="86" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A86" s="10" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B86" s="13">
         <v>46165</v>
@@ -9230,7 +9238,7 @@
         <v>30</v>
       </c>
       <c r="E86" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F86" s="9" t="s">
         <v>43</v>
@@ -9281,7 +9289,7 @@
     </row>
     <row r="87" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A87" s="10" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B87" s="13">
         <v>46165</v>
@@ -9293,7 +9301,7 @@
         <v>30</v>
       </c>
       <c r="E87" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F87" s="9" t="s">
         <v>43</v>
@@ -9344,7 +9352,7 @@
     </row>
     <row r="88" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A88" s="10" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B88" s="13">
         <v>46165</v>
@@ -9356,7 +9364,7 @@
         <v>30</v>
       </c>
       <c r="E88" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F88" s="9" t="s">
         <v>47</v>
@@ -9407,7 +9415,7 @@
     </row>
     <row r="89" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A89" s="10" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B89" s="13">
         <v>46165</v>
@@ -9419,7 +9427,7 @@
         <v>30</v>
       </c>
       <c r="E89" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F89" s="9" t="s">
         <v>47</v>
@@ -9470,7 +9478,7 @@
     </row>
     <row r="90" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A90" s="10" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B90" s="13">
         <v>46165</v>
@@ -9482,7 +9490,7 @@
         <v>30</v>
       </c>
       <c r="E90" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F90" s="9" t="s">
         <v>47</v>
@@ -9533,7 +9541,7 @@
     </row>
     <row r="91" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A91" s="10" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B91" s="13">
         <v>46165</v>
@@ -9545,7 +9553,7 @@
         <v>30</v>
       </c>
       <c r="E91" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F91" s="9" t="s">
         <v>47</v>
@@ -9596,7 +9604,7 @@
     </row>
     <row r="92" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A92" s="10" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B92" s="13">
         <v>46165</v>
@@ -9608,7 +9616,7 @@
         <v>30</v>
       </c>
       <c r="E92" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F92" s="9" t="s">
         <v>47</v>
@@ -9659,7 +9667,7 @@
     </row>
     <row r="93" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A93" s="10" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B93" s="13">
         <v>46165</v>
@@ -9671,7 +9679,7 @@
         <v>30</v>
       </c>
       <c r="E93" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F93" s="9" t="s">
         <v>47</v>
@@ -9722,7 +9730,7 @@
     </row>
     <row r="94" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A94" s="10" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B94" s="13">
         <v>46165</v>
@@ -9734,7 +9742,7 @@
         <v>30</v>
       </c>
       <c r="E94" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F94" s="9" t="s">
         <v>47</v>
@@ -9785,7 +9793,7 @@
     </row>
     <row r="95" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A95" s="10" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B95" s="13">
         <v>46165</v>
@@ -9797,7 +9805,7 @@
         <v>30</v>
       </c>
       <c r="E95" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F95" s="9" t="s">
         <v>47</v>
@@ -9848,7 +9856,7 @@
     </row>
     <row r="96" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A96" s="10" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B96" s="13">
         <v>46165</v>
@@ -9860,7 +9868,7 @@
         <v>30</v>
       </c>
       <c r="E96" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F96" s="9" t="s">
         <v>47</v>
@@ -9911,7 +9919,7 @@
     </row>
     <row r="97" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A97" s="10" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B97" s="13">
         <v>46165</v>
@@ -9923,7 +9931,7 @@
         <v>30</v>
       </c>
       <c r="E97" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F97" s="9" t="s">
         <v>47</v>
@@ -9974,7 +9982,7 @@
     </row>
     <row r="98" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A98" s="10" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B98" s="13">
         <v>46165</v>
@@ -9986,7 +9994,7 @@
         <v>30</v>
       </c>
       <c r="E98" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F98" s="9" t="s">
         <v>47</v>
@@ -10037,7 +10045,7 @@
     </row>
     <row r="99" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A99" s="10" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B99" s="13">
         <v>46165</v>
@@ -10049,7 +10057,7 @@
         <v>30</v>
       </c>
       <c r="E99" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F99" s="9" t="s">
         <v>47</v>
@@ -10100,7 +10108,7 @@
     </row>
     <row r="100" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A100" s="10" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B100" s="13">
         <v>46165</v>
@@ -10112,7 +10120,7 @@
         <v>30</v>
       </c>
       <c r="E100" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F100" s="9" t="s">
         <v>47</v>
@@ -10163,7 +10171,7 @@
     </row>
     <row r="101" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A101" s="10" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B101" s="13">
         <v>46165</v>
@@ -10175,7 +10183,7 @@
         <v>30</v>
       </c>
       <c r="E101" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F101" s="9" t="s">
         <v>47</v>
@@ -10226,7 +10234,7 @@
     </row>
     <row r="102" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A102" s="10" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B102" s="13">
         <v>46165</v>
@@ -10238,7 +10246,7 @@
         <v>30</v>
       </c>
       <c r="E102" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F102" s="9" t="s">
         <v>47</v>
@@ -10289,7 +10297,7 @@
     </row>
     <row r="103" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A103" s="10" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B103" s="13">
         <v>46165</v>
@@ -10301,7 +10309,7 @@
         <v>30</v>
       </c>
       <c r="E103" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F103" s="9" t="s">
         <v>47</v>
@@ -10352,7 +10360,7 @@
     </row>
     <row r="104" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A104" s="10" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B104" s="13">
         <v>46165</v>
@@ -10364,7 +10372,7 @@
         <v>30</v>
       </c>
       <c r="E104" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F104" s="9" t="s">
         <v>47</v>
@@ -10415,7 +10423,7 @@
     </row>
     <row r="105" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A105" s="10" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B105" s="13">
         <v>46165</v>
@@ -10427,7 +10435,7 @@
         <v>30</v>
       </c>
       <c r="E105" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F105" s="9" t="s">
         <v>47</v>
@@ -10478,7 +10486,7 @@
     </row>
     <row r="106" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A106" s="10" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B106" s="13">
         <v>46165</v>
@@ -10490,7 +10498,7 @@
         <v>30</v>
       </c>
       <c r="E106" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F106" s="9" t="s">
         <v>47</v>
@@ -10541,7 +10549,7 @@
     </row>
     <row r="107" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A107" s="10" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B107" s="13">
         <v>46165</v>
@@ -10553,7 +10561,7 @@
         <v>30</v>
       </c>
       <c r="E107" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F107" s="9" t="s">
         <v>47</v>
@@ -10604,7 +10612,7 @@
     </row>
     <row r="108" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A108" s="10" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B108" s="13">
         <v>46165</v>
@@ -10616,7 +10624,7 @@
         <v>30</v>
       </c>
       <c r="E108" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F108" s="9" t="s">
         <v>47</v>
@@ -10667,7 +10675,7 @@
     </row>
     <row r="109" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A109" s="10" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B109" s="13">
         <v>46165</v>
@@ -10679,7 +10687,7 @@
         <v>30</v>
       </c>
       <c r="E109" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F109" s="9" t="s">
         <v>47</v>
@@ -10730,7 +10738,7 @@
     </row>
     <row r="110" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A110" s="10" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B110" s="13">
         <v>46165</v>
@@ -10742,7 +10750,7 @@
         <v>30</v>
       </c>
       <c r="E110" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F110" s="9" t="s">
         <v>47</v>
@@ -10793,7 +10801,7 @@
     </row>
     <row r="111" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A111" s="10" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B111" s="13">
         <v>46165</v>
@@ -10805,7 +10813,7 @@
         <v>30</v>
       </c>
       <c r="E111" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F111" s="9" t="s">
         <v>47</v>
@@ -10856,7 +10864,7 @@
     </row>
     <row r="112" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A112" s="10" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B112" s="13">
         <v>46165</v>
@@ -10868,7 +10876,7 @@
         <v>30</v>
       </c>
       <c r="E112" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F112" s="9" t="s">
         <v>47</v>
@@ -10919,7 +10927,7 @@
     </row>
     <row r="113" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A113" s="10" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B113" s="13">
         <v>46165</v>
@@ -10931,7 +10939,7 @@
         <v>30</v>
       </c>
       <c r="E113" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F113" s="9" t="s">
         <v>47</v>
@@ -10982,7 +10990,7 @@
     </row>
     <row r="114" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A114" s="10" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B114" s="13">
         <v>46165</v>
@@ -10994,7 +11002,7 @@
         <v>30</v>
       </c>
       <c r="E114" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F114" s="9" t="s">
         <v>47</v>
@@ -11045,7 +11053,7 @@
     </row>
     <row r="115" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A115" s="10" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B115" s="13">
         <v>46165</v>
@@ -11057,7 +11065,7 @@
         <v>30</v>
       </c>
       <c r="E115" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F115" s="9" t="s">
         <v>47</v>
@@ -11108,7 +11116,7 @@
     </row>
     <row r="116" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A116" s="10" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B116" s="13">
         <v>46165</v>
@@ -11120,7 +11128,7 @@
         <v>30</v>
       </c>
       <c r="E116" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F116" s="9" t="s">
         <v>47</v>
@@ -11171,7 +11179,7 @@
     </row>
     <row r="117" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A117" s="10" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B117" s="13">
         <v>46165</v>
@@ -11183,7 +11191,7 @@
         <v>30</v>
       </c>
       <c r="E117" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F117" s="9" t="s">
         <v>47</v>
@@ -11234,7 +11242,7 @@
     </row>
     <row r="118" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A118" s="10" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B118" s="13">
         <v>46165</v>
@@ -11246,7 +11254,7 @@
         <v>30</v>
       </c>
       <c r="E118" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F118" s="9" t="s">
         <v>47</v>
@@ -11297,7 +11305,7 @@
     </row>
     <row r="119" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A119" s="10" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B119" s="13">
         <v>46165</v>
@@ -11309,7 +11317,7 @@
         <v>30</v>
       </c>
       <c r="E119" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F119" s="9" t="s">
         <v>47</v>
@@ -11360,7 +11368,7 @@
     </row>
     <row r="120" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A120" s="10" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B120" s="13">
         <v>46165</v>
@@ -11372,7 +11380,7 @@
         <v>30</v>
       </c>
       <c r="E120" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F120" s="9" t="s">
         <v>47</v>
@@ -11423,7 +11431,7 @@
     </row>
     <row r="121" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A121" s="10" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B121" s="13">
         <v>46165</v>
@@ -11435,7 +11443,7 @@
         <v>30</v>
       </c>
       <c r="E121" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F121" s="9" t="s">
         <v>47</v>
@@ -11486,7 +11494,7 @@
     </row>
     <row r="122" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A122" s="10" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B122" s="13">
         <v>46165</v>
@@ -11498,7 +11506,7 @@
         <v>30</v>
       </c>
       <c r="E122" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F122" s="9" t="s">
         <v>47</v>
@@ -11549,7 +11557,7 @@
     </row>
     <row r="123" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A123" s="10" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B123" s="13">
         <v>46165</v>
@@ -11561,7 +11569,7 @@
         <v>30</v>
       </c>
       <c r="E123" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F123" s="9" t="s">
         <v>47</v>
@@ -11612,7 +11620,7 @@
     </row>
     <row r="124" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A124" s="10" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B124" s="13">
         <v>46165</v>
@@ -11624,7 +11632,7 @@
         <v>30</v>
       </c>
       <c r="E124" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F124" s="9" t="s">
         <v>47</v>
@@ -11675,7 +11683,7 @@
     </row>
     <row r="125" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A125" s="10" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B125" s="13">
         <v>46165</v>
@@ -11687,7 +11695,7 @@
         <v>30</v>
       </c>
       <c r="E125" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F125" s="9" t="s">
         <v>47</v>
@@ -11738,7 +11746,7 @@
     </row>
     <row r="126" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A126" s="10" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B126" s="13">
         <v>46165</v>
@@ -11750,7 +11758,7 @@
         <v>30</v>
       </c>
       <c r="E126" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F126" s="9" t="s">
         <v>47</v>
@@ -11801,7 +11809,7 @@
     </row>
     <row r="127" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A127" s="10" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B127" s="13">
         <v>46165</v>
@@ -11813,7 +11821,7 @@
         <v>30</v>
       </c>
       <c r="E127" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F127" s="9" t="s">
         <v>50</v>
@@ -11864,7 +11872,7 @@
     </row>
     <row r="128" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A128" s="10" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B128" s="13">
         <v>46165</v>
@@ -11876,7 +11884,7 @@
         <v>30</v>
       </c>
       <c r="E128" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F128" s="9" t="s">
         <v>50</v>
@@ -11927,7 +11935,7 @@
     </row>
     <row r="129" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A129" s="10" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B129" s="13">
         <v>46165</v>
@@ -11939,7 +11947,7 @@
         <v>30</v>
       </c>
       <c r="E129" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F129" s="9" t="s">
         <v>50</v>
@@ -11990,7 +11998,7 @@
     </row>
     <row r="130" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A130" s="10" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B130" s="13">
         <v>46165</v>
@@ -12002,7 +12010,7 @@
         <v>30</v>
       </c>
       <c r="E130" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F130" s="9" t="s">
         <v>50</v>
@@ -12053,7 +12061,7 @@
     </row>
     <row r="131" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A131" s="10" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B131" s="13">
         <v>46165</v>
@@ -12065,7 +12073,7 @@
         <v>30</v>
       </c>
       <c r="E131" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F131" s="9" t="s">
         <v>50</v>
@@ -12116,7 +12124,7 @@
     </row>
     <row r="132" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A132" s="10" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B132" s="13">
         <v>46165</v>
@@ -12128,7 +12136,7 @@
         <v>30</v>
       </c>
       <c r="E132" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F132" s="9" t="s">
         <v>50</v>
@@ -12179,7 +12187,7 @@
     </row>
     <row r="133" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A133" s="10" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B133" s="13">
         <v>46165</v>
@@ -12191,7 +12199,7 @@
         <v>30</v>
       </c>
       <c r="E133" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F133" s="9" t="s">
         <v>50</v>
@@ -12242,7 +12250,7 @@
     </row>
     <row r="134" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A134" s="10" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B134" s="13">
         <v>46165</v>
@@ -12254,7 +12262,7 @@
         <v>30</v>
       </c>
       <c r="E134" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F134" s="9" t="s">
         <v>50</v>
@@ -12305,7 +12313,7 @@
     </row>
     <row r="135" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A135" s="10" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B135" s="13">
         <v>46165</v>
@@ -12317,7 +12325,7 @@
         <v>30</v>
       </c>
       <c r="E135" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F135" s="9" t="s">
         <v>50</v>
@@ -12368,7 +12376,7 @@
     </row>
     <row r="136" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A136" s="10" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B136" s="13">
         <v>46165</v>
@@ -12380,7 +12388,7 @@
         <v>30</v>
       </c>
       <c r="E136" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F136" s="9" t="s">
         <v>50</v>
@@ -12431,7 +12439,7 @@
     </row>
     <row r="137" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A137" s="10" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B137" s="13">
         <v>46165</v>
@@ -12443,7 +12451,7 @@
         <v>30</v>
       </c>
       <c r="E137" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F137" s="9" t="s">
         <v>50</v>
@@ -12494,7 +12502,7 @@
     </row>
     <row r="138" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A138" s="10" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B138" s="13">
         <v>46165</v>
@@ -12506,7 +12514,7 @@
         <v>30</v>
       </c>
       <c r="E138" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F138" s="9" t="s">
         <v>50</v>
@@ -12557,7 +12565,7 @@
     </row>
     <row r="139" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A139" s="10" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B139" s="13">
         <v>46165</v>
@@ -12569,7 +12577,7 @@
         <v>30</v>
       </c>
       <c r="E139" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F139" s="9" t="s">
         <v>50</v>
@@ -12620,7 +12628,7 @@
     </row>
     <row r="140" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A140" s="10" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B140" s="13">
         <v>46165</v>
@@ -12632,7 +12640,7 @@
         <v>30</v>
       </c>
       <c r="E140" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F140" s="9" t="s">
         <v>50</v>
@@ -12683,7 +12691,7 @@
     </row>
     <row r="141" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A141" s="10" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B141" s="13">
         <v>46165</v>
@@ -12695,7 +12703,7 @@
         <v>30</v>
       </c>
       <c r="E141" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F141" s="9" t="s">
         <v>50</v>
@@ -12746,7 +12754,7 @@
     </row>
     <row r="142" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A142" s="11" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B142" s="14">
         <v>46188</v>
@@ -12758,7 +12766,7 @@
         <v>7</v>
       </c>
       <c r="E142" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F142" s="9" t="s">
         <v>37</v>
@@ -12807,7 +12815,7 @@
     </row>
     <row r="143" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A143" s="11" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B143" s="14">
         <v>46188</v>
@@ -12819,7 +12827,7 @@
         <v>7</v>
       </c>
       <c r="E143" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F143" s="9" t="s">
         <v>41</v>
@@ -12868,7 +12876,7 @@
     </row>
     <row r="144" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A144" s="11" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B144" s="14">
         <v>46188</v>
@@ -12880,7 +12888,7 @@
         <v>7</v>
       </c>
       <c r="E144" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F144" s="9" t="s">
         <v>43</v>
@@ -12931,7 +12939,7 @@
     </row>
     <row r="145" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A145" s="11" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B145" s="14">
         <v>46188</v>
@@ -12943,7 +12951,7 @@
         <v>7</v>
       </c>
       <c r="E145" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F145" s="9" t="s">
         <v>43</v>
@@ -12994,7 +13002,7 @@
     </row>
     <row r="146" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A146" s="11" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B146" s="14">
         <v>46188</v>
@@ -13006,7 +13014,7 @@
         <v>7</v>
       </c>
       <c r="E146" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F146" s="9" t="s">
         <v>43</v>
@@ -13057,7 +13065,7 @@
     </row>
     <row r="147" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A147" s="11" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B147" s="14">
         <v>46188</v>
@@ -13069,7 +13077,7 @@
         <v>7</v>
       </c>
       <c r="E147" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F147" s="9" t="s">
         <v>43</v>
@@ -13120,7 +13128,7 @@
     </row>
     <row r="148" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A148" s="11" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B148" s="14">
         <v>46188</v>
@@ -13132,7 +13140,7 @@
         <v>7</v>
       </c>
       <c r="E148" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F148" s="9" t="s">
         <v>43</v>
@@ -13183,7 +13191,7 @@
     </row>
     <row r="149" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A149" s="11" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B149" s="14">
         <v>46188</v>
@@ -13195,7 +13203,7 @@
         <v>7</v>
       </c>
       <c r="E149" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F149" s="9" t="s">
         <v>43</v>
@@ -13246,7 +13254,7 @@
     </row>
     <row r="150" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A150" s="11" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B150" s="14">
         <v>46188</v>
@@ -13258,7 +13266,7 @@
         <v>7</v>
       </c>
       <c r="E150" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F150" s="9" t="s">
         <v>43</v>
@@ -13309,7 +13317,7 @@
     </row>
     <row r="151" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A151" s="11" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B151" s="14">
         <v>46188</v>
@@ -13321,7 +13329,7 @@
         <v>7</v>
       </c>
       <c r="E151" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F151" s="9" t="s">
         <v>43</v>
@@ -13372,7 +13380,7 @@
     </row>
     <row r="152" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A152" s="11" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B152" s="14">
         <v>46188</v>
@@ -13384,7 +13392,7 @@
         <v>7</v>
       </c>
       <c r="E152" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F152" s="9" t="s">
         <v>43</v>
@@ -13435,7 +13443,7 @@
     </row>
     <row r="153" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A153" s="11" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B153" s="14">
         <v>46188</v>
@@ -13447,7 +13455,7 @@
         <v>7</v>
       </c>
       <c r="E153" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F153" s="9" t="s">
         <v>43</v>
@@ -13498,7 +13506,7 @@
     </row>
     <row r="154" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A154" s="11" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B154" s="14">
         <v>46188</v>
@@ -13510,7 +13518,7 @@
         <v>7</v>
       </c>
       <c r="E154" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F154" s="9" t="s">
         <v>43</v>
@@ -13561,7 +13569,7 @@
     </row>
     <row r="155" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A155" s="11" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B155" s="14">
         <v>46188</v>
@@ -13573,7 +13581,7 @@
         <v>7</v>
       </c>
       <c r="E155" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F155" s="9" t="s">
         <v>43</v>
@@ -13624,7 +13632,7 @@
     </row>
     <row r="156" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A156" s="11" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B156" s="14">
         <v>46188</v>
@@ -13636,7 +13644,7 @@
         <v>7</v>
       </c>
       <c r="E156" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F156" s="9" t="s">
         <v>43</v>
@@ -13687,7 +13695,7 @@
     </row>
     <row r="157" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A157" s="11" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B157" s="14">
         <v>46188</v>
@@ -13699,7 +13707,7 @@
         <v>7</v>
       </c>
       <c r="E157" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F157" s="9" t="s">
         <v>43</v>
@@ -13750,7 +13758,7 @@
     </row>
     <row r="158" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A158" s="11" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B158" s="14">
         <v>46188</v>
@@ -13762,7 +13770,7 @@
         <v>7</v>
       </c>
       <c r="E158" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F158" s="9" t="s">
         <v>47</v>
@@ -13813,7 +13821,7 @@
     </row>
     <row r="159" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A159" s="11" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B159" s="14">
         <v>46188</v>
@@ -13825,7 +13833,7 @@
         <v>7</v>
       </c>
       <c r="E159" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F159" s="9" t="s">
         <v>47</v>
@@ -13876,7 +13884,7 @@
     </row>
     <row r="160" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A160" s="11" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B160" s="14">
         <v>46188</v>
@@ -13888,7 +13896,7 @@
         <v>7</v>
       </c>
       <c r="E160" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F160" s="9" t="s">
         <v>47</v>
@@ -13939,7 +13947,7 @@
     </row>
     <row r="161" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A161" s="11" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B161" s="14">
         <v>46188</v>
@@ -13951,7 +13959,7 @@
         <v>7</v>
       </c>
       <c r="E161" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F161" s="9" t="s">
         <v>47</v>
@@ -14002,7 +14010,7 @@
     </row>
     <row r="162" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A162" s="11" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B162" s="14">
         <v>46188</v>
@@ -14014,7 +14022,7 @@
         <v>7</v>
       </c>
       <c r="E162" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F162" s="9" t="s">
         <v>47</v>
@@ -14065,7 +14073,7 @@
     </row>
     <row r="163" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A163" s="11" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B163" s="14">
         <v>46188</v>
@@ -14077,7 +14085,7 @@
         <v>7</v>
       </c>
       <c r="E163" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F163" s="9" t="s">
         <v>47</v>
@@ -14128,7 +14136,7 @@
     </row>
     <row r="164" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A164" s="11" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B164" s="14">
         <v>46188</v>
@@ -14140,7 +14148,7 @@
         <v>7</v>
       </c>
       <c r="E164" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F164" s="9" t="s">
         <v>47</v>
@@ -14191,7 +14199,7 @@
     </row>
     <row r="165" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A165" s="11" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B165" s="14">
         <v>46188</v>
@@ -14203,7 +14211,7 @@
         <v>7</v>
       </c>
       <c r="E165" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F165" s="9" t="s">
         <v>47</v>
@@ -14254,7 +14262,7 @@
     </row>
     <row r="166" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A166" s="11" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B166" s="14">
         <v>46188</v>
@@ -14266,7 +14274,7 @@
         <v>7</v>
       </c>
       <c r="E166" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F166" s="9" t="s">
         <v>47</v>
@@ -14317,7 +14325,7 @@
     </row>
     <row r="167" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A167" s="11" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B167" s="14">
         <v>46188</v>
@@ -14329,7 +14337,7 @@
         <v>7</v>
       </c>
       <c r="E167" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F167" s="9" t="s">
         <v>47</v>
@@ -14380,7 +14388,7 @@
     </row>
     <row r="168" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A168" s="11" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B168" s="14">
         <v>46188</v>
@@ -14392,7 +14400,7 @@
         <v>7</v>
       </c>
       <c r="E168" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F168" s="9" t="s">
         <v>47</v>
@@ -14443,7 +14451,7 @@
     </row>
     <row r="169" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A169" s="11" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B169" s="14">
         <v>46188</v>
@@ -14455,7 +14463,7 @@
         <v>7</v>
       </c>
       <c r="E169" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F169" s="9" t="s">
         <v>47</v>
@@ -14506,7 +14514,7 @@
     </row>
     <row r="170" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A170" s="11" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B170" s="14">
         <v>46188</v>
@@ -14518,7 +14526,7 @@
         <v>7</v>
       </c>
       <c r="E170" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F170" s="9" t="s">
         <v>47</v>
@@ -14569,7 +14577,7 @@
     </row>
     <row r="171" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A171" s="11" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B171" s="14">
         <v>46188</v>
@@ -14581,7 +14589,7 @@
         <v>7</v>
       </c>
       <c r="E171" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F171" s="9" t="s">
         <v>47</v>
@@ -14632,7 +14640,7 @@
     </row>
     <row r="172" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A172" s="11" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B172" s="14">
         <v>46188</v>
@@ -14644,7 +14652,7 @@
         <v>7</v>
       </c>
       <c r="E172" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F172" s="9" t="s">
         <v>47</v>
@@ -14695,7 +14703,7 @@
     </row>
     <row r="173" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A173" s="11" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B173" s="14">
         <v>46188</v>
@@ -14707,7 +14715,7 @@
         <v>7</v>
       </c>
       <c r="E173" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F173" s="9" t="s">
         <v>47</v>
@@ -14758,7 +14766,7 @@
     </row>
     <row r="174" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A174" s="11" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B174" s="14">
         <v>46188</v>
@@ -14770,7 +14778,7 @@
         <v>7</v>
       </c>
       <c r="E174" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F174" s="9" t="s">
         <v>47</v>
@@ -14821,7 +14829,7 @@
     </row>
     <row r="175" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A175" s="11" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B175" s="14">
         <v>46188</v>
@@ -14833,7 +14841,7 @@
         <v>7</v>
       </c>
       <c r="E175" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F175" s="9" t="s">
         <v>47</v>
@@ -14884,7 +14892,7 @@
     </row>
     <row r="176" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A176" s="11" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B176" s="14">
         <v>46188</v>
@@ -14896,7 +14904,7 @@
         <v>7</v>
       </c>
       <c r="E176" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F176" s="9" t="s">
         <v>47</v>
@@ -14947,7 +14955,7 @@
     </row>
     <row r="177" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A177" s="11" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B177" s="14">
         <v>46188</v>
@@ -14959,7 +14967,7 @@
         <v>7</v>
       </c>
       <c r="E177" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F177" s="9" t="s">
         <v>47</v>
@@ -15010,7 +15018,7 @@
     </row>
     <row r="178" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A178" s="11" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B178" s="14">
         <v>46188</v>
@@ -15022,7 +15030,7 @@
         <v>7</v>
       </c>
       <c r="E178" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F178" s="9" t="s">
         <v>47</v>
@@ -15073,7 +15081,7 @@
     </row>
     <row r="179" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A179" s="11" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B179" s="14">
         <v>46188</v>
@@ -15085,7 +15093,7 @@
         <v>7</v>
       </c>
       <c r="E179" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F179" s="9" t="s">
         <v>47</v>
@@ -15136,7 +15144,7 @@
     </row>
     <row r="180" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A180" s="11" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B180" s="14">
         <v>46188</v>
@@ -15148,7 +15156,7 @@
         <v>7</v>
       </c>
       <c r="E180" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F180" s="9" t="s">
         <v>47</v>
@@ -15199,7 +15207,7 @@
     </row>
     <row r="181" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A181" s="11" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B181" s="14">
         <v>46188</v>
@@ -15211,7 +15219,7 @@
         <v>7</v>
       </c>
       <c r="E181" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F181" s="9" t="s">
         <v>47</v>
@@ -15262,7 +15270,7 @@
     </row>
     <row r="182" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A182" s="11" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B182" s="14">
         <v>46188</v>
@@ -15274,7 +15282,7 @@
         <v>7</v>
       </c>
       <c r="E182" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F182" s="9" t="s">
         <v>47</v>
@@ -15325,7 +15333,7 @@
     </row>
     <row r="183" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A183" s="11" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B183" s="14">
         <v>46188</v>
@@ -15337,7 +15345,7 @@
         <v>7</v>
       </c>
       <c r="E183" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F183" s="9" t="s">
         <v>47</v>
@@ -15388,7 +15396,7 @@
     </row>
     <row r="184" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A184" s="11" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B184" s="14">
         <v>46188</v>
@@ -15400,7 +15408,7 @@
         <v>7</v>
       </c>
       <c r="E184" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F184" s="9" t="s">
         <v>47</v>
@@ -15451,7 +15459,7 @@
     </row>
     <row r="185" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A185" s="11" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B185" s="14">
         <v>46188</v>
@@ -15463,7 +15471,7 @@
         <v>7</v>
       </c>
       <c r="E185" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F185" s="9" t="s">
         <v>47</v>
@@ -15514,7 +15522,7 @@
     </row>
     <row r="186" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A186" s="11" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B186" s="14">
         <v>46188</v>
@@ -15526,7 +15534,7 @@
         <v>7</v>
       </c>
       <c r="E186" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F186" s="9" t="s">
         <v>47</v>
@@ -15577,7 +15585,7 @@
     </row>
     <row r="187" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A187" s="11" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B187" s="14">
         <v>46188</v>
@@ -15589,7 +15597,7 @@
         <v>7</v>
       </c>
       <c r="E187" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F187" s="9" t="s">
         <v>47</v>
@@ -15640,7 +15648,7 @@
     </row>
     <row r="188" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A188" s="11" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B188" s="14">
         <v>46188</v>
@@ -15652,7 +15660,7 @@
         <v>7</v>
       </c>
       <c r="E188" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F188" s="9" t="s">
         <v>47</v>
@@ -15703,7 +15711,7 @@
     </row>
     <row r="189" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A189" s="11" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B189" s="14">
         <v>46188</v>
@@ -15715,7 +15723,7 @@
         <v>7</v>
       </c>
       <c r="E189" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F189" s="9" t="s">
         <v>47</v>
@@ -15766,7 +15774,7 @@
     </row>
     <row r="190" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A190" s="11" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B190" s="14">
         <v>46188</v>
@@ -15778,7 +15786,7 @@
         <v>7</v>
       </c>
       <c r="E190" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F190" s="9" t="s">
         <v>47</v>
@@ -15829,7 +15837,7 @@
     </row>
     <row r="191" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A191" s="11" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B191" s="14">
         <v>46188</v>
@@ -15841,7 +15849,7 @@
         <v>7</v>
       </c>
       <c r="E191" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F191" s="9" t="s">
         <v>47</v>
@@ -15892,7 +15900,7 @@
     </row>
     <row r="192" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A192" s="11" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B192" s="14">
         <v>46188</v>
@@ -15904,7 +15912,7 @@
         <v>7</v>
       </c>
       <c r="E192" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F192" s="9" t="s">
         <v>47</v>
@@ -15955,7 +15963,7 @@
     </row>
     <row r="193" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A193" s="11" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B193" s="14">
         <v>46188</v>
@@ -15967,7 +15975,7 @@
         <v>7</v>
       </c>
       <c r="E193" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F193" s="9" t="s">
         <v>47</v>
@@ -16018,7 +16026,7 @@
     </row>
     <row r="194" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A194" s="11" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B194" s="14">
         <v>46188</v>
@@ -16030,7 +16038,7 @@
         <v>7</v>
       </c>
       <c r="E194" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F194" s="9" t="s">
         <v>47</v>
@@ -16081,7 +16089,7 @@
     </row>
     <row r="195" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A195" s="11" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B195" s="14">
         <v>46188</v>
@@ -16093,7 +16101,7 @@
         <v>7</v>
       </c>
       <c r="E195" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F195" s="9" t="s">
         <v>47</v>
@@ -16144,7 +16152,7 @@
     </row>
     <row r="196" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A196" s="11" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B196" s="14">
         <v>46188</v>
@@ -16156,7 +16164,7 @@
         <v>7</v>
       </c>
       <c r="E196" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F196" s="9" t="s">
         <v>47</v>
@@ -16207,7 +16215,7 @@
     </row>
     <row r="197" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A197" s="11" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B197" s="14">
         <v>46188</v>
@@ -16219,7 +16227,7 @@
         <v>7</v>
       </c>
       <c r="E197" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F197" s="9" t="s">
         <v>50</v>
@@ -16270,7 +16278,7 @@
     </row>
     <row r="198" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A198" s="11" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B198" s="14">
         <v>46188</v>
@@ -16282,7 +16290,7 @@
         <v>7</v>
       </c>
       <c r="E198" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F198" s="9" t="s">
         <v>50</v>
@@ -16333,7 +16341,7 @@
     </row>
     <row r="199" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A199" s="11" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B199" s="14">
         <v>46188</v>
@@ -16345,7 +16353,7 @@
         <v>7</v>
       </c>
       <c r="E199" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F199" s="9" t="s">
         <v>50</v>
@@ -16396,7 +16404,7 @@
     </row>
     <row r="200" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A200" s="11" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B200" s="14">
         <v>46188</v>
@@ -16408,7 +16416,7 @@
         <v>7</v>
       </c>
       <c r="E200" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F200" s="9" t="s">
         <v>50</v>
@@ -16459,7 +16467,7 @@
     </row>
     <row r="201" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A201" s="11" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B201" s="14">
         <v>46188</v>
@@ -16471,7 +16479,7 @@
         <v>7</v>
       </c>
       <c r="E201" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F201" s="9" t="s">
         <v>50</v>
@@ -16522,7 +16530,7 @@
     </row>
     <row r="202" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A202" s="11" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B202" s="14">
         <v>46188</v>
@@ -16534,7 +16542,7 @@
         <v>7</v>
       </c>
       <c r="E202" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F202" s="9" t="s">
         <v>50</v>
@@ -16585,7 +16593,7 @@
     </row>
     <row r="203" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A203" s="11" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B203" s="14">
         <v>46188</v>
@@ -16597,7 +16605,7 @@
         <v>7</v>
       </c>
       <c r="E203" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F203" s="9" t="s">
         <v>50</v>
@@ -16648,7 +16656,7 @@
     </row>
     <row r="204" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A204" s="11" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B204" s="14">
         <v>46188</v>
@@ -16660,7 +16668,7 @@
         <v>7</v>
       </c>
       <c r="E204" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F204" s="9" t="s">
         <v>50</v>
@@ -16711,7 +16719,7 @@
     </row>
     <row r="205" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A205" s="11" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B205" s="14">
         <v>46188</v>
@@ -16723,7 +16731,7 @@
         <v>7</v>
       </c>
       <c r="E205" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F205" s="9" t="s">
         <v>50</v>
@@ -16774,7 +16782,7 @@
     </row>
     <row r="206" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A206" s="11" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B206" s="14">
         <v>46188</v>
@@ -16786,7 +16794,7 @@
         <v>7</v>
       </c>
       <c r="E206" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F206" s="9" t="s">
         <v>50</v>
@@ -16837,7 +16845,7 @@
     </row>
     <row r="207" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A207" s="11" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B207" s="14">
         <v>46188</v>
@@ -16849,7 +16857,7 @@
         <v>7</v>
       </c>
       <c r="E207" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F207" s="9" t="s">
         <v>50</v>
@@ -16900,7 +16908,7 @@
     </row>
     <row r="208" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A208" s="11" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B208" s="14">
         <v>46188</v>
@@ -16912,7 +16920,7 @@
         <v>7</v>
       </c>
       <c r="E208" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F208" s="9" t="s">
         <v>50</v>
@@ -16963,7 +16971,7 @@
     </row>
     <row r="209" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A209" s="11" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B209" s="14">
         <v>46188</v>
@@ -16975,7 +16983,7 @@
         <v>7</v>
       </c>
       <c r="E209" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F209" s="9" t="s">
         <v>50</v>
@@ -17026,7 +17034,7 @@
     </row>
     <row r="210" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A210" s="11" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B210" s="14">
         <v>46188</v>
@@ -17038,7 +17046,7 @@
         <v>7</v>
       </c>
       <c r="E210" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F210" s="9" t="s">
         <v>50</v>
@@ -17089,7 +17097,7 @@
     </row>
     <row r="211" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A211" s="11" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B211" s="14">
         <v>46188</v>
@@ -17101,7 +17109,7 @@
         <v>7</v>
       </c>
       <c r="E211" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F211" s="9" t="s">
         <v>50</v>

</xml_diff>